<commit_message>
feat(testakten): Berlin-Akte Multi-Format-Unterordner ausbauen
emails/ auf fuenf Nachrichten erweitert (Nachlassgericht, Ralf Lohse,
Stadtsparkasse, Jana Lohse). csv/fristen_und_sicherung.csv um weitere
Fristen ergaenzt. xlsx/nachlassinventar_digital_analog.xlsx um
Verkehrswertschaetzung und Massnahmenspalte erweitert. pdfs/ um vier
weitere gerenderte Belege ergaenzt (Kontosperrvermerk, Honorarabrechnung,
Nachlassnotizen-Abschrift, Galerieplattform-Kontoauszug).
</commit_message>
<xml_diff>
--- a/testakten/erbrecht-digitaler-nachlass-passwortsafe-berlin/xlsx/nachlassinventar_digital_analog.xlsx
+++ b/testakten/erbrecht-digitaler-nachlass-passwortsafe-berlin/xlsx/nachlassinventar_digital_analog.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,16 @@
           <t>Streit</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verkehrswert Schaetzung</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Bewertungsgrundlage</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +485,14 @@
           <t>Herausgabe</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Zeitwert IT-Geraet, Marktvergleich</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -500,6 +518,14 @@
           <t>Rechte</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Datenwert nicht bezifferbar, Geraetewert Marktvergleich</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -525,6 +551,14 @@
           <t>Vermächtnis Jana</t>
         </is>
       </c>
+      <c r="F4" t="n">
+        <v>5200</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sammlerwert Kameraboerse</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -548,6 +582,14 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>Erbnachweis</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>7840</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Offene Forderung, Nennwert</t>
         </is>
       </c>
     </row>
@@ -562,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -586,6 +628,11 @@
           <t>Priorität</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Massnahme</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -603,6 +650,11 @@
           <t>hoch</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Rechnungslauf pruefen, ggf. kuendigen</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -620,6 +672,11 @@
           <t>hoch</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Zugriff ueber Bank mit Erbschein beantragen</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -635,6 +692,11 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>mittel</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Abo kuendigen, Galerie-Inhalte sichern</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v432.1.0: Erbrechtsakten als Kanzleivorgaenge ausbauen
</commit_message>
<xml_diff>
--- a/testakten/erbrecht-digitaler-nachlass-passwortsafe-berlin/xlsx/nachlassinventar_digital_analog.xlsx
+++ b/testakten/erbrecht-digitaler-nachlass-passwortsafe-berlin/xlsx/nachlassinventar_digital_analog.xlsx
@@ -8,9 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Konten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Konten und Dienste" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Belegstatus" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventar'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Konten und Dienste'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Belegstatus'!$A$1:$F$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +31,31 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017324D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +63,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00CFD6DA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,186 +445,472 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Ort</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Wertannahme</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ort am Todestag</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ort aktuell</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Wertansatz EUR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Zugriff</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Streit</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Verkehrswert Schaetzung</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Bewertungsgrundlage</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Offene Frage</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Stand</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Studiorechner Mac</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>bei Ralf</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2200</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Studiorechner Mac Pro</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Atelier Veteranenstraße</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>bei Ralf Lohse</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Kaufbeleg 2023</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Ralf</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Herausgabe</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Zeitwert IT-Geraet, Marktvergleich</t>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Seriennummer und Datenträgerzustand</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Sicherung offen</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>NAS Bildarchiv</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Studio</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4800</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NAS mit 18,4 TB Bildarchiv</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Atelier Serverschrank</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Inventur 14.02.2025</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Passwort fehlt</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Rechte</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>4500</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Datenwert nicht bezifferbar, Geraetewert Marktvergleich</t>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Bestand und Rechteketten</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Stromversorgung aktiv</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Leica M10</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Wohnung Eva</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>3900</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Leica M10 mit Objektiv</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Wohnung Kastanienallee</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>bei Eva</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Händlerauskunft 28.06.2026</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Eva</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Vermächtnis Jana</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>5200</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Sammlerwert Kameraboerse</t>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Zuwendung an Jana</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>versiegelt</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Agenturhonorar</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Nordfenster</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Agenturhonorar Nordfenster</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Forderung</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>gesperrt</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>7840</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Abrechnung NF-2026-0518</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Agentur</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Erbnachweis</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>fällig, nicht ausgezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Bildrechte und Lizenzen</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>digital</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>teilweise unzugänglich</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Ertragsdaten 2023 bis 2026</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>ungeklärt</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Verkehrswert und Releases</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Gutachten angefragt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>A-01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Girokonto Stadtsparkasse</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>gesperrt</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Erbnachweis</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>7840</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Offene Forderung, Nennwert</t>
+      <c r="E7" s="2" t="n">
+        <v>34812.44</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Bankauskunft 04.07.2026</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>laufende Lastschriften</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>A-02</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tagesgeld</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>gesperrt</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>12880.16</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Bankauskunft 04.07.2026</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Bestattung</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Verbindlichkeit</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Rechnung bei Eva</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>-8940</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Rechnung Bestattung Klose</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Eva</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Schlussrechnung offen</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Anzahlung 4980,00 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Auftrag Ahlers</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>mögliche Verbindlichkeit</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>-2600</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Auftragsbestätigung</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Kanzlei</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Lieferung oder Rückzahlung</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>noch keine Fälligkeit anerkannt</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -604,103 +921,446 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dienst</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Hinweis</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Priorität</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Massnahme</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Vertragspartner</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kundennummer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kosten</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Nächster Termin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Zugang</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Maßnahme</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Cloudspeicher</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Rechnung im E-Mail-Konto</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>hoch</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Rechnungslauf pruefen, ggf. kuendigen</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cloudwerk Europe</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Armin Lohse</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CW-881402</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>12,00 EUR monatlich</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>15.07.2026</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Bankauszug</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Passwortsafe vermutet</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Datenbestand vor Kündigung sichern</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bank Online</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Passwortsafe vermutet</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>hoch</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Zugriff ueber Bank mit Erbschein beantragen</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Galerieplattform</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Armin Lohse</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GP-204771</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>89,00 EUR jährlich</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>07.07.2026</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Portal-Ausdruck</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Ralf kennt Zugang</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Zugriff protokollieren</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Galerieplattform</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Abo läuft weiter</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>mittel</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Abo kuendigen, Galerie-Inhalte sichern</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Nordfenster Portal</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Armin Lohse</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>NF-3318</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>keine Grundgebühr</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Agenturmail</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Account im Lesemodus</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Erbnachweis abstimmen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Stadtsparkasse Onlinebanking</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Armin Lohse</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>NL-6604-26</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>deaktiviert</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Bankauskunft</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>gesperrt</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>nur über Bank kommunizieren</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unterlage</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ablage</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Vollständig</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nächste Handlung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Testament Original</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>12.09.2021</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Kanzleitresor Fach T</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lohse</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ablieferung koordinieren</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Notizzettel</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>undatiert</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>nur Farbfoto</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ralf Lohse</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Original und Rückseite</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Kaufbeleg Mac Pro</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>16.03.2023</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ordner Studio</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lohse</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Seriennummer abgleichen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Model-Releases Hafenstadt</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2019 bis 2025</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>NAS vermutet</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>teilweise</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Nordfenster</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>fehlende zwei Dateien suchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Vertrag Ahlers</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>11.01.2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Mandantenordner</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lohse</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Lieferumfang prüfen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>